<commit_message>
ksoft - 8180 - 06/03/2026 - Hora: 00:00:00,00
</commit_message>
<xml_diff>
--- a/ksoft/docs/fields_details/BOM_Detail.xlsx
+++ b/ksoft/docs/fields_details/BOM_Detail.xlsx
@@ -916,13 +916,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4C408B1-B491-4798-BEE7-3FB52BBB8E18}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3CB9AB5-9F56-485D-97C2-7786752D9EE1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5EA2762F-3C81-43C6-88E7-40AA10245B89}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E56B888-4D85-4F82-B8F1-CAFC253914E9}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4268222-3321-4539-A25F-41D7678BEDF2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{192445BA-3601-4508-855A-52FDDAB46CBC}"/>
 </file>
</xml_diff>

<commit_message>
ksoft - 8180 - 23/03/2026 00:00:00,00
</commit_message>
<xml_diff>
--- a/ksoft/docs/fields_details/BOM_Detail.xlsx
+++ b/ksoft/docs/fields_details/BOM_Detail.xlsx
@@ -916,13 +916,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3CB9AB5-9F56-485D-97C2-7786752D9EE1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4C408B1-B491-4798-BEE7-3FB52BBB8E18}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E56B888-4D85-4F82-B8F1-CAFC253914E9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5EA2762F-3C81-43C6-88E7-40AA10245B89}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{192445BA-3601-4508-855A-52FDDAB46CBC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4268222-3321-4539-A25F-41D7678BEDF2}"/>
 </file>
</xml_diff>